<commit_message>
feat(core): 7-3a — LiveSystem 결합 + 리허설 판정 루프 (발주 없음)
- 코어 시동 시 LS/HL 접속(bootstrap_live)·리허설 엔진 시작. 접속 실패해도
  API는 계속(화면 조작 가능, 시세만 없음). 로그 콘솔+logs/core_날짜.log
- pair_signal: est 기반 진입/청산 스프레드(주문 화면 표시·판정 공용) —
  진입 = HL매수d(est)−국내매수d, 국내 기준가 SF=이론가/주식=현재가
- RehearsalEngine(core_engine.py): 0.5초 틱, 세트 조건(진입 ≥/청산 ≤ 기준값)
  충족 시 실주문과 동일한 계획·역산가·est 계산 후 로그 기록만. 가상 포지션·
  발주누적(fired_qty)·딜레이·운영시간·세션(데드존) 가드 동일 적용
- /state에 live 스냅샷(신호·현재가·환율·가상포지션·rehearsal 표시)
- 주문 화면: 진입/청산 신호 패널(빨강/파랑)·국내/HL 현재가·환율·현재진입수량
  (/보유최대) 실시간 표시 자리 신설
- 테스트 13종(pair_signal 검산, 판정·딜레이·목표완료·운영시간·가상포지션)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/주문화면0722.xlsx
+++ b/주문화면0722.xlsx
@@ -779,7 +779,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -821,6 +821,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1377,7 +1378,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R116"/>
+  <dimension ref="A1:S116"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12.08203125" customWidth="1"/>
@@ -1389,8 +1390,9 @@
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="11.25" customWidth="1"/>
     <col min="12" max="12" width="11.58203125" customWidth="1"/>
-    <col min="13" max="13" width="10.08203125" customWidth="1"/>
-    <col min="15" max="15" width="11.75" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
+    <col min="14" max="14" width="4.83203125" customWidth="1"/>
+    <col min="16" max="16" width="11.75" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
@@ -1719,7 +1721,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="50" spans="2:18" x14ac:dyDescent="0.45">
+    <row r="50" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B50" s="1" t="s">
         <v>116</v>
       </c>
@@ -1733,15 +1735,16 @@
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
       <c r="L50" s="3"/>
-      <c r="N50" s="1" t="s">
+      <c r="M50" s="29"/>
+      <c r="O50" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="O50" s="2"/>
       <c r="P50" s="2"/>
       <c r="Q50" s="2"/>
-      <c r="R50" s="3"/>
-    </row>
-    <row r="51" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="R50" s="2"/>
+      <c r="S50" s="3"/>
+    </row>
+    <row r="51" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B51" s="4"/>
       <c r="C51" s="14" t="s">
         <v>44</v>
@@ -1757,12 +1760,13 @@
         <v>118</v>
       </c>
       <c r="L51" s="5"/>
-      <c r="N51" s="4" t="s">
+      <c r="M51" s="29"/>
+      <c r="O51" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="R51" s="5"/>
-    </row>
-    <row r="52" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="S51" s="5"/>
+    </row>
+    <row r="52" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B52" s="4"/>
       <c r="C52" s="15" t="s">
         <v>49</v>
@@ -1778,15 +1782,16 @@
       </c>
       <c r="J52" s="16"/>
       <c r="L52" s="5"/>
-      <c r="N52" s="6" t="s">
+      <c r="M52" s="29"/>
+      <c r="O52" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="O52" s="7"/>
       <c r="P52" s="7"/>
       <c r="Q52" s="7"/>
-      <c r="R52" s="8"/>
-    </row>
-    <row r="53" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="R52" s="7"/>
+      <c r="S52" s="8"/>
+    </row>
+    <row r="53" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B53" s="4"/>
       <c r="F53" s="16" t="s">
         <v>27</v>
@@ -1798,29 +1803,33 @@
         <v>-0.01</v>
       </c>
       <c r="L53" s="5"/>
-    </row>
-    <row r="54" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="M53" s="29"/>
+    </row>
+    <row r="54" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B54" s="4"/>
       <c r="L54" s="5"/>
-      <c r="N54" t="s">
+      <c r="M54" s="29"/>
+      <c r="O54" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="55" spans="2:18" x14ac:dyDescent="0.45">
+    <row r="55" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B55" s="4"/>
       <c r="C55" t="s">
         <v>120</v>
       </c>
       <c r="L55" s="5"/>
-    </row>
-    <row r="56" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="M55" s="29"/>
+    </row>
+    <row r="56" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B56" s="4"/>
       <c r="C56" s="18" t="s">
         <v>52</v>
       </c>
       <c r="L56" s="5"/>
-    </row>
-    <row r="57" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="M56" s="29"/>
+    </row>
+    <row r="57" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B57" s="4"/>
       <c r="C57" s="16" t="s">
         <v>107</v>
@@ -1850,11 +1859,12 @@
         <v>60</v>
       </c>
       <c r="L57" s="5"/>
-      <c r="N57" t="s">
+      <c r="M57" s="29"/>
+      <c r="O57" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="58" spans="2:18" x14ac:dyDescent="0.45">
+    <row r="58" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B58" s="20" t="s">
         <v>61</v>
       </c>
@@ -1876,11 +1886,12 @@
       <c r="J58" s="16"/>
       <c r="K58" s="16"/>
       <c r="L58" s="5"/>
-      <c r="N58" t="s">
+      <c r="M58" s="29"/>
+      <c r="O58" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="59" spans="2:18" x14ac:dyDescent="0.45">
+    <row r="59" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B59" s="20" t="s">
         <v>63</v>
       </c>
@@ -1900,11 +1911,12 @@
       <c r="J59" s="16"/>
       <c r="K59" s="16"/>
       <c r="L59" s="5"/>
-      <c r="N59" t="s">
+      <c r="M59" s="29"/>
+      <c r="O59" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="60" spans="2:18" x14ac:dyDescent="0.45">
+    <row r="60" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B60" s="20" t="s">
         <v>64</v>
       </c>
@@ -1924,19 +1936,22 @@
       <c r="J60" s="16"/>
       <c r="K60" s="16"/>
       <c r="L60" s="5"/>
-    </row>
-    <row r="61" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="M60" s="29"/>
+    </row>
+    <row r="61" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B61" s="4"/>
       <c r="L61" s="5"/>
-    </row>
-    <row r="62" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="M61" s="29"/>
+    </row>
+    <row r="62" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B62" s="4"/>
       <c r="C62" s="18" t="s">
         <v>65</v>
       </c>
       <c r="L62" s="5"/>
-    </row>
-    <row r="63" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="M62" s="29"/>
+    </row>
+    <row r="63" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B63" s="4"/>
       <c r="C63" s="16" t="s">
         <v>119</v>
@@ -1966,11 +1981,12 @@
         <v>68</v>
       </c>
       <c r="L63" s="5"/>
-      <c r="N63" t="s">
+      <c r="M63" s="29"/>
+      <c r="O63" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="64" spans="2:18" x14ac:dyDescent="0.45">
+    <row r="64" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B64" s="20" t="s">
         <v>61</v>
       </c>
@@ -1992,13 +2008,14 @@
       <c r="J64" s="16"/>
       <c r="K64" s="16"/>
       <c r="L64" s="5"/>
-      <c r="N64" s="22" t="s">
+      <c r="M64" s="29"/>
+      <c r="O64" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="O64" s="22"/>
       <c r="P64" s="22"/>
-    </row>
-    <row r="65" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="Q64" s="22"/>
+    </row>
+    <row r="65" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B65" s="20" t="s">
         <v>63</v>
       </c>
@@ -2018,8 +2035,9 @@
       <c r="J65" s="16"/>
       <c r="K65" s="16"/>
       <c r="L65" s="5"/>
-    </row>
-    <row r="66" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M65" s="29"/>
+    </row>
+    <row r="66" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B66" s="20" t="s">
         <v>64</v>
       </c>
@@ -2039,11 +2057,12 @@
       <c r="J66" s="16"/>
       <c r="K66" s="16"/>
       <c r="L66" s="5"/>
-      <c r="N66" t="s">
+      <c r="M66" s="29"/>
+      <c r="O66" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="67" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="67" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B67" s="6"/>
       <c r="C67" s="7"/>
       <c r="D67" s="7"/>
@@ -2055,8 +2074,9 @@
       <c r="J67" s="7"/>
       <c r="K67" s="7"/>
       <c r="L67" s="8"/>
-    </row>
-    <row r="70" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M67" s="29"/>
+    </row>
+    <row r="70" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B70" s="10" t="s">
         <v>104</v>
       </c>
@@ -2072,7 +2092,7 @@
       <c r="F70" s="12"/>
       <c r="G70" s="13"/>
     </row>
-    <row r="72" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="72" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B72" s="1" t="s">
         <v>115</v>
       </c>
@@ -2086,8 +2106,9 @@
       <c r="J72" s="2"/>
       <c r="K72" s="2"/>
       <c r="L72" s="3"/>
-    </row>
-    <row r="73" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M72" s="29"/>
+    </row>
+    <row r="73" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B73" s="4"/>
       <c r="C73" s="14" t="s">
         <v>44</v>
@@ -2108,11 +2129,12 @@
       <c r="L73" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="M73" t="s">
+      <c r="M73" s="29"/>
+      <c r="N73" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="74" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="74" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B74" s="4"/>
       <c r="C74" s="15" t="s">
         <v>49</v>
@@ -2129,11 +2151,12 @@
       <c r="I74" s="16"/>
       <c r="J74" s="16"/>
       <c r="L74" s="16"/>
-      <c r="M74" t="s">
+      <c r="M74" s="29"/>
+      <c r="N74" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="75" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="75" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B75" s="4"/>
       <c r="F75" s="16" t="s">
         <v>27</v>
@@ -2147,32 +2170,36 @@
       <c r="I75" s="16"/>
       <c r="J75" s="16"/>
       <c r="L75" s="5"/>
-      <c r="M75" t="s">
+      <c r="M75" s="29"/>
+      <c r="N75" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="76" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="76" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B76" s="4"/>
       <c r="L76" s="5"/>
-    </row>
-    <row r="77" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M76" s="29"/>
+    </row>
+    <row r="77" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B77" s="4"/>
       <c r="L77" s="5"/>
-      <c r="M77" t="s">
+      <c r="M77" s="29"/>
+      <c r="N77" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="78" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="78" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B78" s="4"/>
       <c r="C78" s="18" t="s">
         <v>52</v>
       </c>
       <c r="L78" s="5"/>
-      <c r="M78" t="s">
+      <c r="M78" s="29"/>
+      <c r="N78" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="79" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="79" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B79" s="4"/>
       <c r="C79" s="19" t="s">
         <v>108</v>
@@ -2199,8 +2226,9 @@
         <v>110</v>
       </c>
       <c r="L79" s="5"/>
-    </row>
-    <row r="80" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M79" s="29"/>
+    </row>
+    <row r="80" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B80" s="20" t="s">
         <v>61</v>
       </c>
@@ -2221,11 +2249,12 @@
       <c r="I80" s="16"/>
       <c r="J80" s="16"/>
       <c r="L80" s="5"/>
-      <c r="M80" t="s">
+      <c r="M80" s="29"/>
+      <c r="N80" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="81" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B81" s="20" t="s">
         <v>63</v>
       </c>
@@ -2244,8 +2273,9 @@
       <c r="I81" s="16"/>
       <c r="J81" s="16"/>
       <c r="L81" s="5"/>
-    </row>
-    <row r="82" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M81" s="29"/>
+    </row>
+    <row r="82" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B82" s="20" t="s">
         <v>64</v>
       </c>
@@ -2264,22 +2294,25 @@
       <c r="I82" s="16"/>
       <c r="J82" s="16"/>
       <c r="L82" s="5"/>
-      <c r="M82" t="s">
+      <c r="M82" s="29"/>
+      <c r="N82" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="83" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="83" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B83" s="4"/>
       <c r="L83" s="5"/>
-    </row>
-    <row r="84" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M83" s="29"/>
+    </row>
+    <row r="84" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B84" s="4"/>
       <c r="C84" s="18" t="s">
         <v>65</v>
       </c>
       <c r="L84" s="5"/>
-    </row>
-    <row r="85" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M84" s="29"/>
+    </row>
+    <row r="85" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B85" s="4"/>
       <c r="C85" s="19" t="s">
         <v>109</v>
@@ -2306,8 +2339,9 @@
         <v>111</v>
       </c>
       <c r="L85" s="5"/>
-    </row>
-    <row r="86" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M85" s="29"/>
+    </row>
+    <row r="86" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B86" s="20" t="s">
         <v>61</v>
       </c>
@@ -2328,8 +2362,9 @@
       <c r="I86" s="16"/>
       <c r="J86" s="16"/>
       <c r="L86" s="5"/>
-    </row>
-    <row r="87" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M86" s="29"/>
+    </row>
+    <row r="87" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B87" s="20" t="s">
         <v>63</v>
       </c>
@@ -2348,8 +2383,9 @@
       <c r="I87" s="16"/>
       <c r="J87" s="16"/>
       <c r="L87" s="5"/>
-    </row>
-    <row r="88" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M87" s="29"/>
+    </row>
+    <row r="88" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B88" s="20" t="s">
         <v>64</v>
       </c>
@@ -2368,8 +2404,9 @@
       <c r="I88" s="16"/>
       <c r="J88" s="16"/>
       <c r="L88" s="5"/>
-    </row>
-    <row r="89" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M88" s="29"/>
+    </row>
+    <row r="89" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B89" s="6"/>
       <c r="C89" s="7"/>
       <c r="D89" s="7"/>
@@ -2381,18 +2418,19 @@
       <c r="J89" s="7"/>
       <c r="K89" s="7"/>
       <c r="L89" s="8"/>
-    </row>
-    <row r="92" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M89" s="29"/>
+    </row>
+    <row r="92" spans="2:14" x14ac:dyDescent="0.45">
       <c r="C92" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="93" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="93" spans="2:14" x14ac:dyDescent="0.45">
       <c r="C93" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="96" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="96" spans="2:14" x14ac:dyDescent="0.45">
       <c r="C96" t="s">
         <v>83</v>
       </c>

</xml_diff>